<commit_message>
Update AP, Add color
</commit_message>
<xml_diff>
--- a/assets/floor_3_data.xlsx
+++ b/assets/floor_3_data.xlsx
@@ -70,9 +70,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -404,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -428,6 +427,9 @@
       <c r="G1" t="str">
         <v>LastAudit</v>
       </c>
+      <c r="H1" t="str">
+        <v>Color</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -451,6 +453,9 @@
       <c r="G2" t="str">
         <v/>
       </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -474,6 +479,9 @@
       <c r="G3" t="str">
         <v/>
       </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -497,6 +505,9 @@
       <c r="G4" t="str">
         <v/>
       </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -520,17 +531,20 @@
       <c r="G5" t="str">
         <v/>
       </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -554,132 +568,228 @@
       <c r="G1" t="str">
         <v>LastAudit</v>
       </c>
+      <c r="H1" t="str">
+        <v>Color</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>WIFI-AP-Lobby</v>
+        <v>THMJNCHOTH01S05</v>
       </c>
       <c r="B2" t="str">
-        <v>AP</v>
+        <v>Switch</v>
       </c>
       <c r="C2">
-        <v>-800</v>
+        <v>-1111</v>
       </c>
       <c r="D2">
-        <v>1200</v>
+        <v>38</v>
       </c>
       <c r="E2" t="str">
-        <v>Main entrance access point</v>
+        <v>Office Switch</v>
       </c>
       <c r="F2" t="str">
         <v>Active</v>
       </c>
-      <c r="G2" s="1">
-        <v>44927</v>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v>Orange</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>WIFI-AP-Canteen</v>
+        <v>AP09c</v>
       </c>
       <c r="B3" t="str">
         <v>AP</v>
       </c>
       <c r="C3">
-        <v>550</v>
+        <v>-2349</v>
       </c>
       <c r="D3">
-        <v>900</v>
+        <v>-413</v>
       </c>
       <c r="E3" t="str">
-        <v>Cafeteria coverage</v>
+        <v>Main entrance access point</v>
       </c>
       <c r="F3" t="str">
-        <v>Inactive</v>
+        <v>Active</v>
       </c>
       <c r="G3" t="str">
         <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>Salmon</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>SRV-DC-01</v>
+        <v>AP10c</v>
       </c>
       <c r="B4" t="str">
-        <v>Server</v>
+        <v>AP</v>
       </c>
       <c r="C4">
-        <v>-1500</v>
+        <v>-1978</v>
       </c>
       <c r="D4">
-        <v>-1300</v>
+        <v>-393</v>
       </c>
       <c r="E4" t="str">
-        <v>Domain Controller 1</v>
+        <v>Cafeteria coverage</v>
       </c>
       <c r="F4" t="str">
         <v>Active</v>
       </c>
       <c r="G4" t="str">
         <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>Salmon</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>SRV-FS-01</v>
+        <v>AP11c</v>
       </c>
       <c r="B5" t="str">
-        <v>Server</v>
+        <v>AP</v>
       </c>
       <c r="C5">
-        <v>-1550</v>
+        <v>-1841</v>
       </c>
       <c r="D5">
-        <v>-1300</v>
+        <v>113</v>
       </c>
       <c r="E5" t="str">
-        <v>File Server 1</v>
+        <v/>
       </c>
       <c r="F5" t="str">
         <v>Active</v>
       </c>
-      <c r="G5" s="1">
-        <v>44927</v>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v>Salmon</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>SW-IDF-01</v>
+        <v>AP12c</v>
       </c>
       <c r="B6" t="str">
-        <v>Switch</v>
+        <v>AP</v>
       </c>
       <c r="C6">
-        <v>-1450</v>
+        <v>-2010</v>
       </c>
       <c r="D6">
-        <v>-1350</v>
+        <v>172</v>
       </c>
       <c r="E6" t="str">
-        <v>Main Distribution Frame Switch</v>
+        <v/>
       </c>
       <c r="F6" t="str">
         <v>Active</v>
       </c>
       <c r="G6" t="str">
         <v/>
+      </c>
+      <c r="H6" t="str">
+        <v>Salmon</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>AP13c</v>
+      </c>
+      <c r="B7" t="str">
+        <v>AP</v>
+      </c>
+      <c r="C7">
+        <v>-2548</v>
+      </c>
+      <c r="D7">
+        <v>574</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v>Salmon</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>AP14c</v>
+      </c>
+      <c r="B8" t="str">
+        <v>AP</v>
+      </c>
+      <c r="C8">
+        <v>-2200</v>
+      </c>
+      <c r="D8">
+        <v>676</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v>Salmon</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>AP15c</v>
+      </c>
+      <c r="B9" t="str">
+        <v>AP</v>
+      </c>
+      <c r="C9">
+        <v>-2383</v>
+      </c>
+      <c r="D9">
+        <v>286</v>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v>Active</v>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v>Salmon</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -703,6 +813,9 @@
       <c r="G1" t="str">
         <v>LastAudit</v>
       </c>
+      <c r="H1" t="str">
+        <v>Color</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -726,6 +839,9 @@
       <c r="G2" t="str">
         <v/>
       </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -749,6 +865,9 @@
       <c r="G3" t="str">
         <v/>
       </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -772,17 +891,20 @@
       <c r="G4" t="str">
         <v/>
       </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -806,6 +928,9 @@
       <c r="G1" t="str">
         <v>LastAudit</v>
       </c>
+      <c r="H1" t="str">
+        <v>Color</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -829,17 +954,20 @@
       <c r="G2" t="str">
         <v>2025-12-15</v>
       </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -863,6 +991,9 @@
       <c r="G1" t="str">
         <v>LastAudit</v>
       </c>
+      <c r="H1" t="str">
+        <v>Color</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -886,6 +1017,9 @@
       <c r="G2" t="str">
         <v/>
       </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -909,6 +1043,9 @@
       <c r="G3" t="str">
         <v/>
       </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -932,6 +1069,9 @@
       <c r="G4" t="str">
         <v/>
       </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -955,17 +1095,20 @@
       <c r="G5" t="str">
         <v>2025-12-15</v>
       </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -989,6 +1132,9 @@
       <c r="G1" t="str">
         <v>LastAudit</v>
       </c>
+      <c r="H1" t="str">
+        <v>Color</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1012,6 +1158,9 @@
       <c r="G2" t="str">
         <v/>
       </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -1035,6 +1184,9 @@
       <c r="G3" t="str">
         <v/>
       </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -1058,17 +1210,20 @@
       <c r="G4" t="str">
         <v/>
       </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1092,6 +1247,9 @@
       <c r="G1" t="str">
         <v>LastAudit</v>
       </c>
+      <c r="H1" t="str">
+        <v>Color</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1115,6 +1273,9 @@
       <c r="G2" t="str">
         <v>2025-12-15</v>
       </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -1138,10 +1299,13 @@
       <c r="G3" t="str">
         <v>2025-12-15</v>
       </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>